<commit_message>
feat: password reset, account deletion, Google sign-in
</commit_message>
<xml_diff>
--- a/4Prep_3-Month-Plan.xlsx
+++ b/4Prep_3-Month-Plan.xlsx
@@ -23,9 +23,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="ddd, mmm d"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="ddd, mmm d"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -167,7 +166,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -196,7 +195,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -226,6 +225,9 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -616,7 +618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C21"/>
+  <dimension ref="B1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -624,6 +626,7 @@
     <col width="95" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -645,6 +648,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="B6" s="4" t="inlineStr"/>
       <c r="C6" s="5" t="inlineStr"/>
@@ -802,6 +806,18 @@
       <c r="C21" s="5" t="inlineStr">
         <is>
           <t>Fits only if weeks 1–3 hold. If Φ is hard or the paper is ambiguous (R5), weeks 2–3 slip and eat the buffer — which is why they're front-loaded. If you slip, cut universities (10 not 20), NEVER the safeguards.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>AI COUNSELOR</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Structured only — NO chatbot (decided 2026-07-24). The counselor speaks through the Pathway Generator + the 5 tools as sourced cards, kept honest by the claim validator + designed refusal states. Built in Week 6 (real Claude output replaces the hardcoded text in the existing AIResponseBlock cards) and hardened in Week 8 (golden-set grounding check). Deliberately no chat window — nothing invites a question you have no sourced answer for.</t>
         </is>
       </c>
     </row>
@@ -895,12 +911,12 @@
       <c r="E2" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F2" s="12" t="n">
+      <c r="F2" s="24" t="n">
         <v>46230</v>
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H2" s="13" t="inlineStr">
@@ -933,12 +949,12 @@
       <c r="E3" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F3" s="12" t="n">
+      <c r="F3" s="24" t="n">
         <v>46230</v>
       </c>
       <c r="G3" s="11" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="H3" s="13" t="inlineStr">
@@ -971,7 +987,7 @@
       <c r="E4" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="F4" s="12" t="n">
+      <c r="F4" s="24" t="n">
         <v>46233</v>
       </c>
       <c r="G4" s="11" t="inlineStr">
@@ -1005,7 +1021,7 @@
       <c r="E5" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F5" s="12" t="n">
+      <c r="F5" s="24" t="n">
         <v>46234</v>
       </c>
       <c r="G5" s="11" t="inlineStr">
@@ -1043,7 +1059,7 @@
       <c r="E6" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="12" t="n">
+      <c r="F6" s="24" t="n">
         <v>46236</v>
       </c>
       <c r="G6" s="11" t="inlineStr">
@@ -1077,7 +1093,7 @@
       <c r="E7" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="F7" s="12" t="n">
+      <c r="F7" s="24" t="n">
         <v>46239</v>
       </c>
       <c r="G7" s="11" t="inlineStr">
@@ -1115,7 +1131,7 @@
       <c r="E8" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F8" s="12" t="n">
+      <c r="F8" s="24" t="n">
         <v>46240</v>
       </c>
       <c r="G8" s="11" t="inlineStr">
@@ -1149,7 +1165,7 @@
       <c r="E9" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F9" s="12" t="n">
+      <c r="F9" s="24" t="n">
         <v>46242</v>
       </c>
       <c r="G9" s="11" t="inlineStr">
@@ -1183,7 +1199,7 @@
       <c r="E10" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F10" s="12" t="n">
+      <c r="F10" s="24" t="n">
         <v>46243</v>
       </c>
       <c r="G10" s="11" t="inlineStr">
@@ -1217,7 +1233,7 @@
       <c r="E11" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="F11" s="12" t="n">
+      <c r="F11" s="24" t="n">
         <v>46246</v>
       </c>
       <c r="G11" s="11" t="inlineStr">
@@ -1251,7 +1267,7 @@
       <c r="E12" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="F12" s="12" t="n">
+      <c r="F12" s="24" t="n">
         <v>46248</v>
       </c>
       <c r="G12" s="11" t="inlineStr">
@@ -1289,7 +1305,7 @@
       <c r="E13" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F13" s="12" t="n">
+      <c r="F13" s="24" t="n">
         <v>46249</v>
       </c>
       <c r="G13" s="11" t="inlineStr">
@@ -1327,7 +1343,7 @@
       <c r="E14" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F14" s="12" t="n">
+      <c r="F14" s="24" t="n">
         <v>46250</v>
       </c>
       <c r="G14" s="11" t="inlineStr">
@@ -1361,7 +1377,7 @@
       <c r="E15" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F15" s="12" t="n">
+      <c r="F15" s="24" t="n">
         <v>46251</v>
       </c>
       <c r="G15" s="11" t="inlineStr">
@@ -1395,7 +1411,7 @@
       <c r="E16" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F16" s="12" t="n">
+      <c r="F16" s="24" t="n">
         <v>46253</v>
       </c>
       <c r="G16" s="11" t="inlineStr">
@@ -1429,7 +1445,7 @@
       <c r="E17" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="F17" s="12" t="n">
+      <c r="F17" s="24" t="n">
         <v>46256</v>
       </c>
       <c r="G17" s="11" t="inlineStr">
@@ -1463,7 +1479,7 @@
       <c r="E18" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F18" s="12" t="n">
+      <c r="F18" s="24" t="n">
         <v>46257</v>
       </c>
       <c r="G18" s="11" t="inlineStr">
@@ -1501,7 +1517,7 @@
       <c r="E19" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="F19" s="12" t="n">
+      <c r="F19" s="24" t="n">
         <v>46262</v>
       </c>
       <c r="G19" s="11" t="inlineStr">
@@ -1535,7 +1551,7 @@
       <c r="E20" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F20" s="12" t="n">
+      <c r="F20" s="24" t="n">
         <v>46263</v>
       </c>
       <c r="G20" s="11" t="inlineStr">
@@ -1569,7 +1585,7 @@
       <c r="E21" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F21" s="12" t="n">
+      <c r="F21" s="24" t="n">
         <v>46264</v>
       </c>
       <c r="G21" s="11" t="inlineStr">
@@ -1592,18 +1608,18 @@
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>The grounded AI counselor (CORE)</t>
+          <t>The AI counselor — grounded, structured (no chatbot)</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>Wire Claude API Pathway Generator: profile + records + Φ + citation IDs → structured, sourced narrative</t>
+          <t>AI counselor: write the prompt + wire the Claude API (profile + record bundle + Φ + citation IDs → structured JSON pathway) and render it into the existing AIResponseBlock cards (Results + Pathway Generator). No free-text facts.</t>
         </is>
       </c>
       <c r="E22" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="F22" s="12" t="n">
+      <c r="F22" s="24" t="n">
         <v>46268</v>
       </c>
       <c r="G22" s="11" t="inlineStr">
@@ -1613,7 +1629,7 @@
       </c>
       <c r="H22" s="13" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>CORE · structured-only, no chat window</t>
         </is>
       </c>
     </row>
@@ -1630,18 +1646,18 @@
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>The grounded AI counselor (CORE)</t>
+          <t>The AI counselor — grounded, structured (no chatbot)</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>Build the claim validator: strip any figure/name/deadline with no citation; missing fact → say so</t>
+          <t>Build the claim validator: strip any figure/name/deadline with no citation ID; on a missing required fact, return an honest refusal instead of a guess.</t>
         </is>
       </c>
       <c r="E23" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="F23" s="12" t="n">
+      <c r="F23" s="24" t="n">
         <v>46271</v>
       </c>
       <c r="G23" s="11" t="inlineStr">
@@ -1651,7 +1667,7 @@
       </c>
       <c r="H23" s="13" t="inlineStr">
         <is>
-          <t>Non-negotiable safeguard</t>
+          <t>The safeguard that keeps the counselor honest</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1695,7 @@
       <c r="E24" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F24" s="12" t="n">
+      <c r="F24" s="24" t="n">
         <v>46273</v>
       </c>
       <c r="G24" s="11" t="inlineStr">
@@ -1717,7 +1733,7 @@
       <c r="E25" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="F25" s="12" t="n">
+      <c r="F25" s="24" t="n">
         <v>46276</v>
       </c>
       <c r="G25" s="11" t="inlineStr">
@@ -1751,7 +1767,7 @@
       <c r="E26" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F26" s="12" t="n">
+      <c r="F26" s="24" t="n">
         <v>46278</v>
       </c>
       <c r="G26" s="11" t="inlineStr">
@@ -1789,7 +1805,7 @@
       <c r="E27" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="F27" s="12" t="n">
+      <c r="F27" s="24" t="n">
         <v>46281</v>
       </c>
       <c r="G27" s="11" t="inlineStr">
@@ -1823,7 +1839,7 @@
       <c r="E28" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F28" s="12" t="n">
+      <c r="F28" s="24" t="n">
         <v>46283</v>
       </c>
       <c r="G28" s="11" t="inlineStr">
@@ -1857,7 +1873,7 @@
       <c r="E29" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F29" s="12" t="n">
+      <c r="F29" s="24" t="n">
         <v>46284</v>
       </c>
       <c r="G29" s="11" t="inlineStr">
@@ -1895,7 +1911,7 @@
       <c r="E30" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F30" s="12" t="n">
+      <c r="F30" s="24" t="n">
         <v>46285</v>
       </c>
       <c r="G30" s="11" t="inlineStr">
@@ -1933,7 +1949,7 @@
       <c r="E31" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="F31" s="12" t="n">
+      <c r="F31" s="24" t="n">
         <v>46288</v>
       </c>
       <c r="G31" s="11" t="inlineStr">
@@ -1967,7 +1983,7 @@
       <c r="E32" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F32" s="12" t="n">
+      <c r="F32" s="24" t="n">
         <v>46289</v>
       </c>
       <c r="G32" s="11" t="inlineStr">
@@ -2001,7 +2017,7 @@
       <c r="E33" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F33" s="12" t="n">
+      <c r="F33" s="24" t="n">
         <v>46290</v>
       </c>
       <c r="G33" s="11" t="inlineStr">
@@ -2035,7 +2051,7 @@
       <c r="E34" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F34" s="12" t="n">
+      <c r="F34" s="24" t="n">
         <v>46292</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
@@ -2069,7 +2085,7 @@
       <c r="E35" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F35" s="12" t="n">
+      <c r="F35" s="24" t="n">
         <v>46294</v>
       </c>
       <c r="G35" s="11" t="inlineStr">
@@ -2103,7 +2119,7 @@
       <c r="E36" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F36" s="12" t="n">
+      <c r="F36" s="24" t="n">
         <v>46296</v>
       </c>
       <c r="G36" s="11" t="inlineStr">
@@ -2137,7 +2153,7 @@
       <c r="E37" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F37" s="12" t="n">
+      <c r="F37" s="24" t="n">
         <v>46298</v>
       </c>
       <c r="G37" s="11" t="inlineStr">
@@ -2171,7 +2187,7 @@
       <c r="E38" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F38" s="12" t="n">
+      <c r="F38" s="24" t="n">
         <v>46299</v>
       </c>
       <c r="G38" s="11" t="inlineStr">
@@ -2205,7 +2221,7 @@
       <c r="E39" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F39" s="12" t="n">
+      <c r="F39" s="24" t="n">
         <v>46300</v>
       </c>
       <c r="G39" s="11" t="inlineStr">
@@ -2239,7 +2255,7 @@
       <c r="E40" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="F40" s="12" t="n">
+      <c r="F40" s="24" t="n">
         <v>46302</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
@@ -2273,7 +2289,7 @@
       <c r="E41" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="F41" s="12" t="n">
+      <c r="F41" s="24" t="n">
         <v>46305</v>
       </c>
       <c r="G41" s="11" t="inlineStr">
@@ -2307,7 +2323,7 @@
       <c r="E42" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F42" s="12" t="n">
+      <c r="F42" s="24" t="n">
         <v>46306</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
@@ -2345,7 +2361,7 @@
       <c r="E43" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="F43" s="12" t="n">
+      <c r="F43" s="24" t="n">
         <v>46310</v>
       </c>
       <c r="G43" s="11" t="inlineStr">
@@ -2379,7 +2395,7 @@
       <c r="E44" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F44" s="12" t="n">
+      <c r="F44" s="24" t="n">
         <v>46312</v>
       </c>
       <c r="G44" s="11" t="inlineStr">
@@ -2413,7 +2429,7 @@
       <c r="E45" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F45" s="12" t="n">
+      <c r="F45" s="24" t="n">
         <v>46313</v>
       </c>
       <c r="G45" s="11" t="inlineStr">
@@ -2423,6 +2439,7 @@
       </c>
       <c r="H45" s="13" t="inlineStr"/>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="D47" s="16" t="inlineStr">
         <is>
@@ -2770,17 +2787,17 @@
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>The grounded AI counselor (core)</t>
+          <t>The AI counselor — grounded, structured cards (no chatbot)</t>
         </is>
       </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
-          <t>One real profile → a grounded, sourced pathway</t>
+          <t>One real profile → a grounded, sourced pathway written by Claude into the existing cards</t>
         </is>
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>A deliberately missing figure is provably stripped (red-team once)</t>
+          <t>A deliberately missing figure is provably stripped by the validator (red-team once); no chat window exists</t>
         </is>
       </c>
       <c r="G7" s="11" t="n">
@@ -3520,7 +3537,7 @@
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
     </row>
@@ -3594,7 +3611,7 @@
       </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>